<commit_message>
Daily job digest update (2026-09-18)
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Digest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -652,10 +652,60 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>kubernetes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Golang Kubernetes Engineer</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Arango</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Remote (verify region/visa terms on listing)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16T19:00:02+00:00</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>RemoteOK</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-golang-kubernetes-engineer-arango-1137400</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:J5"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"No,Applied,Interviewing,Rejected,Not Interested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Daily job digest update (2026-10-05)
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>aws, docker, ci/cd, git, jenkins, react</t>
+          <t>linux</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>DevOps Engineer</t>
+          <t>Junior Site Reliability Engineer (SRE) L3</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Wed, 08 Jul 2026 16:41:06 GMT</t>
+          <t>Mon, 24 Aug 2026 12:41:23 GMT</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://wuzzuf.net/jobs/p/75fd08e8-6be9-4821-88c7-d5827171c8e4-DevOps-Engineer-Bright-Creations-Giza-Egypt</t>
+          <t>https://wuzzuf.net/jobs/p/7c073f86-afc0-4c85-9dee-c0ef1bc6943c-Junior-Site-Reliability-Engineer-SRE-L3-Vertex-Technologies-Cairo-Egypt</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -605,45 +605,45 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>linux</t>
+          <t>kubernetes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Junior Site Reliability Engineer (SRE) L3</t>
+          <t>Golang Kubernetes Engineer</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>See listing</t>
+          <t>Arango</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Cairo/Giza area</t>
+          <t>Remote (verify region/visa terms on listing)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 12:41:23 GMT</t>
+          <t>2026-09-16T19:00:02+00:00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Wuzzuf</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://wuzzuf.net/jobs/p/7c073f86-afc0-4c85-9dee-c0ef1bc6943c-Junior-Site-Reliability-Engineer-SRE-L3-Vertex-Technologies-Cairo-Egypt</t>
+          <t>https://remoteOK.com/remote-jobs/remote-golang-kubernetes-engineer-arango-1137400</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -655,45 +655,23 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>kubernetes</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Golang Kubernetes Engineer</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Arango</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Remote (verify region/visa terms on listing)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16T19:00:02+00:00</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>RemoteOK</t>
-        </is>
-      </c>
+          <t>(not refetched this run)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-golang-kubernetes-engineer-arango-1137400</t>
+          <t>https://wuzzuf.net/jobs/p/75fd08e8-6be9-4821-88c7-d5827171c8e4-DevOps-Engineer-Bright-Creations-Giza-Egypt</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily job digest update (2026-10-31)
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Digest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -555,45 +555,45 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>linux</t>
+          <t>terraform, ci/cd, kubernetes, prometheus, grafana, git</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Junior Site Reliability Engineer (SRE) L3</t>
+          <t>Cloud Engineer Automation</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>See listing</t>
+          <t>Smile Digital Health</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Cairo/Giza area</t>
+          <t>Remote (verify region/visa terms on listing)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Mon, 24 Aug 2026 12:41:23 GMT</t>
+          <t>2026-10-29T16:00:03+00:00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Wuzzuf</t>
+          <t>RemoteOK</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://wuzzuf.net/jobs/p/7c073f86-afc0-4c85-9dee-c0ef1bc6943c-Junior-Site-Reliability-Engineer-SRE-L3-Vertex-Technologies-Cairo-Egypt</t>
+          <t>https://remoteOK.com/remote-jobs/remote-cloud-engineer-automation-smile-digital-health-1137600</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -605,45 +605,45 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>kubernetes</t>
+          <t>linux</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Golang Kubernetes Engineer</t>
+          <t>Junior Site Reliability Engineer (SRE) L3</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Arango</t>
+          <t>See listing</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Remote (verify region/visa terms on listing)</t>
+          <t>Cairo/Giza area</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T19:00:02+00:00</t>
+          <t>Mon, 24 Aug 2026 12:41:23 GMT</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>RemoteOK</t>
+          <t>Wuzzuf</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://remoteOK.com/remote-jobs/remote-golang-kubernetes-engineer-arango-1137400</t>
+          <t>https://wuzzuf.net/jobs/p/7c073f86-afc0-4c85-9dee-c0ef1bc6943c-Junior-Site-Reliability-Engineer-SRE-L3-Vertex-Technologies-Cairo-Egypt</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -655,35 +655,85 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>kubernetes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Golang Kubernetes Engineer</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Arango</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Remote (verify region/visa terms on listing)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16T19:00:02+00:00</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>RemoteOK</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://remoteOK.com/remote-jobs/remote-golang-kubernetes-engineer-arango-1137400</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>(not refetched this run)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>https://wuzzuf.net/jobs/p/75fd08e8-6be9-4821-88c7-d5827171c8e4-DevOps-Engineer-Bright-Creations-Giza-Egypt</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"No,Applied,Interviewing,Rejected,Not Interested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>